<commit_message>
feat: add initial contact datasets for birthday automation
</commit_message>
<xml_diff>
--- a/data/data-copy.xlsx
+++ b/data/data-copy.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,52 +417,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>PhoneNumber</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Birthday</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Anniversary</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Classification</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Brief</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Enabled</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>LastSent</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>MessageTemplate</t>
         </is>
@@ -486,8 +474,10 @@
           <t>S K Pattanayak</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>919439809787</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>+919439809787</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -514,8 +504,10 @@
           <t>Villa No. 4 Blue Bell Gyana Vihar, Burla</t>
         </is>
       </c>
-      <c r="H2" t="b">
-        <v>1</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -526,8 +518,10 @@
           <t>Pitambar Mahapatra</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>918917462553</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>+918917462553</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -554,8 +548,10 @@
           <t>Flat No-203, GD Towers Opp HKD Railway Station</t>
         </is>
       </c>
-      <c r="H3" t="b">
-        <v>1</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -566,8 +562,10 @@
           <t>C R Mohapatra</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>919861045797</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>+919861045797</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -594,8 +592,10 @@
           <t>C-11, Near Cancer Ward, Burla</t>
         </is>
       </c>
-      <c r="H4" t="b">
-        <v>1</v>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -606,8 +606,10 @@
           <t>S.K. Swain</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>919937082348</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>+919937082348</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -626,8 +628,10 @@
           <t>Qr No-5 R/6, VSSUT, Burla</t>
         </is>
       </c>
-      <c r="H5" t="b">
-        <v>1</v>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -638,8 +642,10 @@
           <t>P C Naik</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>919437050373</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>+919437050373</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -666,8 +672,10 @@
           <t>HIG - 18, SDA Colony, Mahanadi Encl, Burla</t>
         </is>
       </c>
-      <c r="H6" t="b">
-        <v>1</v>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -678,8 +686,10 @@
           <t>Kalu Charan Swain</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>919937062699</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>+919937062699</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -706,8 +716,10 @@
           <t>6, Udra, Apparment, Sourav Vihar, Burla</t>
         </is>
       </c>
-      <c r="H7" t="b">
-        <v>1</v>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -718,8 +730,10 @@
           <t>M K Mishra</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>919437057186</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>+919437057186</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -746,8 +760,10 @@
           <t>Friends Colony, Burla</t>
         </is>
       </c>
-      <c r="H8" t="b">
-        <v>1</v>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -758,8 +774,10 @@
           <t>Sribasta.K. Mohapatra</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>919437025626</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>+919437025626</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -786,8 +804,10 @@
           <t>Qr.No. C-7, SBI line</t>
         </is>
       </c>
-      <c r="H9" t="b">
-        <v>1</v>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -798,8 +818,10 @@
           <t>S S Kabli</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>919437419983</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>+919437419983</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -826,8 +848,10 @@
           <t>Contractors' Colony, Burla</t>
         </is>
       </c>
-      <c r="H10" t="b">
-        <v>1</v>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -838,8 +862,10 @@
           <t>S. Mahapatra</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>919861255899</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>+919861255899</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -866,8 +892,10 @@
           <t>Sadeipali, New Colony</t>
         </is>
       </c>
-      <c r="H11" t="b">
-        <v>1</v>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -878,8 +906,10 @@
           <t>A T Rout</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>919861065355</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>+919861065355</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -906,8 +936,10 @@
           <t>Hig-20, Mahanadi Enclave, SDA Colony, Burla - 768018</t>
         </is>
       </c>
-      <c r="H12" t="b">
-        <v>1</v>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -918,8 +950,10 @@
           <t>A K Behera</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>919439660204</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>+919439660204</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -946,8 +980,10 @@
           <t>Duplex No.6, Blue Bell Villa, Gyan Vihar</t>
         </is>
       </c>
-      <c r="H13" t="b">
-        <v>1</v>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -958,8 +994,10 @@
           <t>B M Mishra</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>919437050270</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>+919437050270</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -986,8 +1024,10 @@
           <t>Friends' Colony Phandichowk, Burla</t>
         </is>
       </c>
-      <c r="H14" t="b">
-        <v>1</v>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -998,8 +1038,10 @@
           <t>Ashok Nayak</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>919437257983</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>+919437257983</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1026,8 +1068,10 @@
           <t>H No.323 Hills View, near CWC Office, Burla</t>
         </is>
       </c>
-      <c r="H15" t="b">
-        <v>1</v>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1038,8 +1082,10 @@
           <t>B B Panda</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>919437055123</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>+919437055123</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1066,8 +1112,10 @@
           <t>5R/4, Doctors' Colony, Burla</t>
         </is>
       </c>
-      <c r="H16" t="b">
-        <v>1</v>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1078,8 +1126,10 @@
           <t>Sharmila. Garnaik</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>919937367087</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>+919937367087</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1102,8 +1152,10 @@
           <t>Qr. No. C/5 New Doctors' Colony</t>
         </is>
       </c>
-      <c r="H17" t="b">
-        <v>1</v>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1114,8 +1166,10 @@
           <t>K Jena</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>919437055999</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>+919437055999</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1142,8 +1196,10 @@
           <t>Utkal Foundry &amp; Engg. Co Ltd., Remed</t>
         </is>
       </c>
-      <c r="H18" t="b">
-        <v>1</v>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1154,8 +1210,10 @@
           <t>D.K. Mahalik</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>919861134018</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>+919861134018</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1182,8 +1240,10 @@
           <t>6, Udra, Apparment, Sourav Vihar, Burla</t>
         </is>
       </c>
-      <c r="H19" t="b">
-        <v>1</v>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1194,8 +1254,10 @@
           <t>J.N. Mohapatra</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>919861242178</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>+919861242178</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1222,8 +1284,10 @@
           <t>Golgunda</t>
         </is>
       </c>
-      <c r="H20" t="b">
-        <v>1</v>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1234,8 +1298,10 @@
           <t>Nayan Kumar Patel</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>918658920357</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>+918658920357</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1262,8 +1328,10 @@
           <t>Doctor Colony Qr. No. 3R/5 Vimsar</t>
         </is>
       </c>
-      <c r="H21" t="b">
-        <v>1</v>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1274,8 +1342,10 @@
           <t>D.K. Thakur</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>919437401704</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>+919437401704</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1302,8 +1372,10 @@
           <t>Near 41 Block Burla</t>
         </is>
       </c>
-      <c r="H22" t="b">
-        <v>1</v>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1314,8 +1386,10 @@
           <t>Sumanta Nayak</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>917205266049</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>+917205266049</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1342,8 +1416,10 @@
           <t>Near Satya Narayan Villa</t>
         </is>
       </c>
-      <c r="H23" t="b">
-        <v>1</v>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1354,8 +1430,10 @@
           <t>P K Behera</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>919437093574</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>+919437093574</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1382,8 +1460,10 @@
           <t>303, Siba, Brijdham Society, GM, Univ Road</t>
         </is>
       </c>
-      <c r="H24" t="b">
-        <v>1</v>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1394,8 +1474,10 @@
           <t>R C Acharya</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>918249479229</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>+918249479229</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1422,8 +1504,10 @@
           <t>Sai Lodge, Burla</t>
         </is>
       </c>
-      <c r="H25" t="b">
-        <v>1</v>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1434,8 +1518,10 @@
           <t>S C Panda</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>919437257875</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>+919437257875</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1462,8 +1548,10 @@
           <t>C-2, New Doctors' Colony, Burla</t>
         </is>
       </c>
-      <c r="H26" t="b">
-        <v>1</v>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1474,8 +1562,10 @@
           <t>Rashmi Kanta Pati</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>919827763885</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>+919827763885</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1502,8 +1592,10 @@
           <t>JTQ-6 N. Campus, SU</t>
         </is>
       </c>
-      <c r="H27" t="b">
-        <v>1</v>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1514,8 +1606,10 @@
           <t>R K Jajodia</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>919437051257</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>+919437051257</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1542,8 +1636,10 @@
           <t>Gupta Nursing Home, Burla</t>
         </is>
       </c>
-      <c r="H28" t="b">
-        <v>1</v>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -1554,8 +1650,10 @@
           <t>Roshni Kujur</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>918895286201</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>+918895286201</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1574,8 +1672,10 @@
           <t>Qr. No.C/16 Jyotivihar</t>
         </is>
       </c>
-      <c r="H29" t="b">
-        <v>1</v>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -1586,8 +1686,10 @@
           <t>Shashi Bhusan Biswal</t>
         </is>
       </c>
-      <c r="B30" t="n">
-        <v>919337640488</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>+919337640488</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1610,8 +1712,10 @@
           <t>Qr. No.C/5 New Doctors' Colony</t>
         </is>
       </c>
-      <c r="H30" t="b">
-        <v>1</v>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -1622,8 +1726,10 @@
           <t>Subhranshu Dwibedi</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>917008568406</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>+917008568406</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1650,8 +1756,10 @@
           <t>Qr. C-8, PG Chowk Burla</t>
         </is>
       </c>
-      <c r="H31" t="b">
-        <v>1</v>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -1662,8 +1770,10 @@
           <t>D Kapani</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>919337301824</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>+919337301824</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1690,8 +1800,10 @@
           <t>Contractors' Colony, Burla</t>
         </is>
       </c>
-      <c r="H32" t="b">
-        <v>1</v>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -1702,8 +1814,10 @@
           <t>K. K Gupta</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>919348414501</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>+919348414501</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1730,8 +1844,10 @@
           <t>Krishna Niwas Sourav Vihar</t>
         </is>
       </c>
-      <c r="H33" t="b">
-        <v>1</v>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -1742,8 +1858,10 @@
           <t>D Mishra</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>919861086999</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>+919861086999</t>
+        </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1770,8 +1888,10 @@
           <t>4R/3, UCE Colony, Burla</t>
         </is>
       </c>
-      <c r="H34" t="b">
-        <v>1</v>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -1782,8 +1902,10 @@
           <t>B K Dutta</t>
         </is>
       </c>
-      <c r="B35" t="n">
-        <v>919337333013</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>+919337333013</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1810,8 +1932,10 @@
           <t>Brooks Hill Sakhipara, SBP</t>
         </is>
       </c>
-      <c r="H35" t="b">
-        <v>1</v>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
@@ -1822,8 +1946,10 @@
           <t>S P Padhi</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>919437050571</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>+919437050571</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1850,8 +1976,10 @@
           <t>Contractors' Colony, Burla</t>
         </is>
       </c>
-      <c r="H36" t="b">
-        <v>1</v>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -1862,8 +1990,10 @@
           <t>Sudhir Sahu</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>919938883353</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>+919938883353</t>
+        </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1890,8 +2020,10 @@
           <t>Qr. No.C-7 Near P.G.Chowk</t>
         </is>
       </c>
-      <c r="H37" t="b">
-        <v>1</v>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
@@ -1902,8 +2034,10 @@
           <t>Dinesh Nayak</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>917978938512</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>+917978938512</t>
+        </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1930,8 +2064,10 @@
           <t>H no-12, Udra Comp. Sourav Bihar, Burla</t>
         </is>
       </c>
-      <c r="H38" t="b">
-        <v>1</v>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -1942,8 +2078,10 @@
           <t>B. Behuria</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>919437084140</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>+919437084140</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1970,8 +2108,10 @@
           <t>D-20, Jagruti Vihar MCL, Burla</t>
         </is>
       </c>
-      <c r="H39" t="b">
-        <v>1</v>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -1982,8 +2122,10 @@
           <t>Bulu Maharana</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>919438439068</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>+919438439068</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -2010,8 +2152,10 @@
           <t>P.G. Dept. Lib. &amp; Inf. Sc. SU</t>
         </is>
       </c>
-      <c r="H40" t="b">
-        <v>1</v>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -2022,8 +2166,10 @@
           <t>M.R. Mahanand</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>919439536915</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>+919439536915</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -2050,8 +2196,10 @@
           <t>STQ-6, North Camp. Jyoti Vihar</t>
         </is>
       </c>
-      <c r="H41" t="b">
-        <v>1</v>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
@@ -2062,8 +2210,10 @@
           <t>B K Tripathy</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>919861087533</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>+919861087533</t>
+        </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -2090,8 +2240,10 @@
           <t>Contractor's Colony Burla</t>
         </is>
       </c>
-      <c r="H42" t="b">
-        <v>1</v>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -2102,8 +2254,10 @@
           <t>Shaswat Sarangi</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>919861443600</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>+919861443600</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -2130,8 +2284,10 @@
           <t>Sourav Vihar, Burla</t>
         </is>
       </c>
-      <c r="H43" t="b">
-        <v>1</v>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>

</xml_diff>